<commit_message>
Movilidad con IPC a 2 decimales y descarga de resultados en todos los notebooks
- ANSES actualiza el haber con la variacion del IPC(t-2) calculada desde los niveles
  con 2 decimales (error 0 en 29/29 meses; con la publicada a 1 decimal llegaba a
  0,05 p.p.). Corrige contrafactual IIJP (+0,77% en sep-26) y costo fiscal; los
  indices no cambian. Control de la regla con tolerancia 0,005 p.p.
- src/exportar.py: Excel, graficos y CSV. Cada notebook termina descargando un ZIP
  con todo (escribe en _descargas/, no toca data/processed ni output/).
- NB02: test estadistico con 3 decimales y ponderaciones efectivas en %.
- Docs actualizadas (README, revision_TP, ESTADO, CONTEXTO, CLAUDE).
</commit_message>
<xml_diff>
--- a/output/IIJP_resultados.xlsx
+++ b/output/IIJP_resultados.xlsx
@@ -464,7 +464,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ultimo IPC: 2026-08 | ultimo haber: 2026-09 | ultima IMIG: 2026-08</t>
+          <t>Ultimo IPC: 2026-08 | ultimo haber: 2026-09 | ultima IMIG: 2026-08 | replicas bootstrap: 500</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Montos fiscales en millones de pesos corrientes. Ver README y docs/ para la metodologia.</t>
+          <t>Montos fiscales en millones de pesos corrientes. Metodologia: README y docs/ del repo github.com/santiagoriverti/IPC_jubilados.</t>
         </is>
       </c>
     </row>
@@ -9212,10 +9212,10 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>119244.264</v>
+        <v>119254.8353</v>
       </c>
       <c r="I87" t="n">
-        <v>119561.403</v>
+        <v>119550.8317</v>
       </c>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="n">
@@ -9256,10 +9256,10 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>149651.55132</v>
+        <v>149629.04185091</v>
       </c>
       <c r="I88" t="n">
-        <v>151006.051989</v>
+        <v>151004.65552027</v>
       </c>
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="n">
@@ -9300,10 +9300,10 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>180479.77089192</v>
+        <v>180467.5873763825</v>
       </c>
       <c r="I89" t="n">
-        <v>183321.347114646</v>
+        <v>183334.7522671598</v>
       </c>
       <c r="J89" t="n">
         <v>70000</v>
@@ -9352,13 +9352,13 @@
         <v>1</v>
       </c>
       <c r="H90" t="n">
-        <v>204303.1006496535</v>
+        <v>204361.4959450155</v>
       </c>
       <c r="I90" t="n">
-        <v>208619.6930164671</v>
+        <v>208653.2815552546</v>
       </c>
       <c r="J90" t="n">
-        <v>79240.00000000001</v>
+        <v>79268</v>
       </c>
       <c r="K90" t="n">
         <v>82731.69424653072</v>
@@ -9395,22 +9395,22 @@
         <v>260141.6</v>
       </c>
       <c r="E91" t="n">
-        <v>190124.4741</v>
+        <v>190141.602431</v>
       </c>
       <c r="F91" t="n">
-        <v>189953.19079</v>
+        <v>189987.447452</v>
       </c>
       <c r="G91" t="n">
-        <v>0.999099099099099</v>
+        <v>0.999189262228628</v>
       </c>
       <c r="H91" t="n">
-        <v>226776.4417211154</v>
+        <v>226861.6966485618</v>
       </c>
       <c r="I91" t="n">
-        <v>231359.239555262</v>
+        <v>231438.2199010884</v>
       </c>
       <c r="J91" t="n">
-        <v>87956.40000000002</v>
+        <v>87995.40680000001</v>
       </c>
       <c r="K91" t="n">
         <v>88158.6492245984</v>
@@ -9447,22 +9447,22 @@
         <v>276931.1</v>
       </c>
       <c r="E92" t="n">
-        <v>206855.4278208</v>
+        <v>206931.1059256573</v>
       </c>
       <c r="F92" t="n">
-        <v>207618.83753347</v>
+        <v>207694.2775545264</v>
       </c>
       <c r="G92" t="n">
-        <v>1.003690547164812</v>
+        <v>1.00368804692487</v>
       </c>
       <c r="H92" t="n">
-        <v>246732.7685925736</v>
+        <v>246893.5844626298</v>
       </c>
       <c r="I92" t="n">
-        <v>252875.6488339014</v>
+        <v>253008.2619958698</v>
       </c>
       <c r="J92" t="n">
-        <v>95696.56320000003</v>
+        <v>95765.40122044002</v>
       </c>
       <c r="K92" t="n">
         <v>91743.87907408943</v>
@@ -9499,22 +9499,22 @@
         <v>285580.82</v>
       </c>
       <c r="E93" t="n">
-        <v>215543.3557892737</v>
+        <v>215580.8261533498</v>
       </c>
       <c r="F93" t="n">
-        <v>215923.5910348088</v>
+        <v>215918.9709456856</v>
       </c>
       <c r="G93" t="n">
-        <v>1.001764077784457</v>
+        <v>1.00156852906805</v>
       </c>
       <c r="H93" t="n">
-        <v>257095.5448734617</v>
+        <v>257213.7362931677</v>
       </c>
       <c r="I93" t="n">
-        <v>262990.6747872574</v>
+        <v>263027.3891709062</v>
       </c>
       <c r="J93" t="n">
-        <v>99715.81885440004</v>
+        <v>99768.39499145442</v>
       </c>
       <c r="K93" t="n">
         <v>91875.34506393042</v>
@@ -9551,22 +9551,22 @@
         <v>295454.42</v>
       </c>
       <c r="E94" t="n">
-        <v>225458.3501555803</v>
+        <v>225454.4279911732</v>
       </c>
       <c r="F94" t="n">
-        <v>226071.9998134448</v>
+        <v>226110.346374322</v>
       </c>
       <c r="G94" t="n">
-        <v>1.002721787227845</v>
+        <v>1.002909316924902</v>
       </c>
       <c r="H94" t="n">
-        <v>268921.9399376409</v>
+        <v>268994.1254153948</v>
       </c>
       <c r="I94" t="n">
-        <v>275351.2365022585</v>
+        <v>275442.2819397729</v>
       </c>
       <c r="J94" t="n">
-        <v>104302.7465217024</v>
+        <v>104337.787482063</v>
       </c>
       <c r="K94" t="n">
         <v>92234.94546660256</v>
@@ -9603,22 +9603,22 @@
         <v>304540.23</v>
       </c>
       <c r="E95" t="n">
-        <v>234476.6841618035</v>
+        <v>234540.2414392175</v>
       </c>
       <c r="F95" t="n">
-        <v>235340.951805796</v>
+        <v>235380.8705756692</v>
       </c>
       <c r="G95" t="n">
-        <v>1.003685942792487</v>
+        <v>1.003584157376548</v>
       </c>
       <c r="H95" t="n">
-        <v>279678.8175351465</v>
+        <v>279834.5886696352</v>
       </c>
       <c r="I95" t="n">
-        <v>286640.6371988511</v>
+        <v>286735.4154993036</v>
       </c>
       <c r="J95" t="n">
-        <v>108474.8563825705</v>
+        <v>108542.6003175902</v>
       </c>
       <c r="K95" t="n">
         <v>92734.84624735358</v>
@@ -9655,22 +9655,22 @@
         <v>314320.56</v>
       </c>
       <c r="E96" t="n">
-        <v>244324.7048965992</v>
+        <v>244320.5695072329</v>
       </c>
       <c r="F96" t="n">
-        <v>245225.2717816394</v>
+        <v>245337.48140102</v>
       </c>
       <c r="G96" t="n">
-        <v>1.003685942792487</v>
+        <v>1.004162203353725</v>
       </c>
       <c r="H96" t="n">
-        <v>291425.3278716227</v>
+        <v>291503.691017159</v>
       </c>
       <c r="I96" t="n">
-        <v>298679.5439612028</v>
+        <v>298864.3235749241</v>
       </c>
       <c r="J96" t="n">
-        <v>113030.8003506385</v>
+        <v>113068.8267508337</v>
       </c>
       <c r="K96" t="n">
         <v>94069.77953254395</v>
@@ -9707,22 +9707,22 @@
         <v>322798.48</v>
       </c>
       <c r="E97" t="n">
-        <v>252876.0695679802</v>
+        <v>252798.4932691339</v>
       </c>
       <c r="F97" t="n">
-        <v>253562.9310222152</v>
+        <v>253777.090761215</v>
       </c>
       <c r="G97" t="n">
-        <v>1.002716197920224</v>
+        <v>1.003871057455391</v>
       </c>
       <c r="H97" t="n">
-        <v>301625.2143471295</v>
+        <v>301618.8690954545</v>
       </c>
       <c r="I97" t="n">
-        <v>308834.6484558837</v>
+        <v>309145.2563059015</v>
       </c>
       <c r="J97" t="n">
-        <v>116986.8783629109</v>
+        <v>116992.3150390876</v>
       </c>
       <c r="K97" t="n">
         <v>95028.0921528269</v>
@@ -9759,22 +9759,22 @@
         <v>329598.76</v>
       </c>
       <c r="E98" t="n">
-        <v>259703.7234463156</v>
+        <v>259598.7727380735</v>
       </c>
       <c r="F98" t="n">
-        <v>260155.5672287928</v>
+        <v>260476.8059573111</v>
       </c>
       <c r="G98" t="n">
-        <v>1.001739843297128</v>
+        <v>1.003382270301114</v>
       </c>
       <c r="H98" t="n">
-        <v>309769.0951345019</v>
+        <v>309732.4166741222</v>
       </c>
       <c r="I98" t="n">
-        <v>316864.3493157367</v>
+        <v>317306.6910723773</v>
       </c>
       <c r="J98" t="n">
-        <v>120145.5240787094</v>
+        <v>120139.4083136391</v>
       </c>
       <c r="K98" t="n">
         <v>95015.03747717013</v>
@@ -9811,22 +9811,22 @@
         <v>335907.01</v>
       </c>
       <c r="E99" t="n">
-        <v>265936.6128090272</v>
+        <v>265907.0229156087</v>
       </c>
       <c r="F99" t="n">
-        <v>266399.3008422838</v>
+        <v>266702.2016196909</v>
       </c>
       <c r="G99" t="n">
-        <v>1.001739843297128</v>
+        <v>1.002990438896134</v>
       </c>
       <c r="H99" t="n">
-        <v>317203.55341773</v>
+        <v>317258.9143993033</v>
       </c>
       <c r="I99" t="n">
-        <v>324469.0936993144</v>
+        <v>324890.3209890071</v>
       </c>
       <c r="J99" t="n">
-        <v>123029.0166565985</v>
+        <v>123058.7959356605</v>
       </c>
       <c r="K99" t="n">
         <v>95218.57453527581</v>
@@ -9863,22 +9863,22 @@
         <v>343086.5</v>
       </c>
       <c r="E100" t="n">
-        <v>273116.9013548709</v>
+        <v>273086.5125343301</v>
       </c>
       <c r="F100" t="n">
-        <v>273592.0819650255</v>
+        <v>273929.8312835845</v>
       </c>
       <c r="G100" t="n">
-        <v>1.001739843297128</v>
+        <v>1.003088101061558</v>
       </c>
       <c r="H100" t="n">
-        <v>325768.0493600087</v>
+        <v>325824.9050880845</v>
       </c>
       <c r="I100" t="n">
-        <v>333229.7592291959</v>
+        <v>333694.8486878092</v>
       </c>
       <c r="J100" t="n">
-        <v>126350.8001063266</v>
+        <v>126381.3834259233</v>
       </c>
       <c r="K100" t="n">
         <v>95496.01775153728</v>
@@ -9915,22 +9915,22 @@
         <v>349121.71</v>
       </c>
       <c r="E101" t="n">
-        <v>279125.4731846781</v>
+        <v>279121.7244613388</v>
       </c>
       <c r="F101" t="n">
-        <v>279611.107768256</v>
+        <v>280038.4665212084</v>
       </c>
       <c r="G101" t="n">
-        <v>1.001739843297128</v>
+        <v>1.003284380897398</v>
       </c>
       <c r="H101" t="n">
-        <v>332934.9464459289</v>
+        <v>333025.6354905311</v>
       </c>
       <c r="I101" t="n">
-        <v>340560.8139322382</v>
+        <v>341136.2438135473</v>
       </c>
       <c r="J101" t="n">
-        <v>129130.5177086658</v>
+        <v>129174.4119996362</v>
       </c>
       <c r="K101" t="n">
         <v>94097.27622214259</v>
@@ -9967,22 +9967,22 @@
         <v>355820.63</v>
       </c>
       <c r="E102" t="n">
-        <v>285824.4845411104</v>
+        <v>285820.645848411</v>
       </c>
       <c r="F102" t="n">
-        <v>286601.3854624624</v>
+        <v>287095.4358775428</v>
       </c>
       <c r="G102" t="n">
-        <v>1.002718104862847</v>
+        <v>1.004460104781262</v>
       </c>
       <c r="H102" t="n">
-        <v>340925.3851606312</v>
+        <v>341018.2507423038</v>
       </c>
       <c r="I102" t="n">
-        <v>349074.8342805441</v>
+        <v>349732.8771576487</v>
       </c>
       <c r="J102" t="n">
-        <v>132229.6501336738</v>
+        <v>132274.5978876275</v>
       </c>
       <c r="K102" t="n">
         <v>93748.6153997815</v>
@@ -10019,22 +10019,22 @@
         <v>366481.74</v>
       </c>
       <c r="E103" t="n">
-        <v>296399.9904691314</v>
+        <v>296481.7559385567</v>
       </c>
       <c r="F103" t="n">
-        <v>296345.8325681862</v>
+        <v>296827.9711537915</v>
       </c>
       <c r="G103" t="n">
-        <v>0.9998172810300717</v>
+        <v>1.00116774542885</v>
       </c>
       <c r="H103" t="n">
-        <v>353539.6244115746</v>
+        <v>353738.2314949918</v>
       </c>
       <c r="I103" t="n">
-        <v>360943.3786460827</v>
+        <v>361588.821693293</v>
       </c>
       <c r="J103" t="n">
-        <v>137122.1471886197</v>
+        <v>137208.440388836</v>
       </c>
       <c r="K103" t="n">
         <v>95807.26774995995</v>
@@ -10071,22 +10071,22 @@
         <v>374723.93</v>
       </c>
       <c r="E104" t="n">
-        <v>304699.1902022671</v>
+        <v>304723.9487536486</v>
       </c>
       <c r="F104" t="n">
-        <v>304347.1700475272</v>
+        <v>304693.912389367</v>
       </c>
       <c r="G104" t="n">
-        <v>0.9988446961263459</v>
+        <v>0.999901430903595</v>
       </c>
       <c r="H104" t="n">
-        <v>363438.7338950987</v>
+        <v>363572.1543305526</v>
       </c>
       <c r="I104" t="n">
-        <v>370688.8498695269</v>
+        <v>371170.9254681653</v>
       </c>
       <c r="J104" t="n">
-        <v>140961.5673099011</v>
+        <v>141022.8350316456</v>
       </c>
       <c r="K104" t="n">
         <v>96901.9394185229</v>
@@ -10123,22 +10123,22 @@
         <v>379294.79</v>
       </c>
       <c r="E105" t="n">
-        <v>309269.6780553011</v>
+        <v>309294.8079849533</v>
       </c>
       <c r="F105" t="n">
-        <v>309216.7247682876</v>
+        <v>309416.6680314022</v>
       </c>
       <c r="G105" t="n">
-        <v>0.9998287795708054</v>
+        <v>1.000393993184828</v>
       </c>
       <c r="H105" t="n">
-        <v>368890.3149035251</v>
+        <v>369025.7366455109</v>
       </c>
       <c r="I105" t="n">
-        <v>376619.8714674393</v>
+        <v>376924.0748129218</v>
       </c>
       <c r="J105" t="n">
-        <v>143075.9908195496</v>
+        <v>143138.1775571203</v>
       </c>
       <c r="K105" t="n">
         <v>96519.96436079894</v>
@@ -10175,22 +10175,22 @@
         <v>384305.37</v>
       </c>
       <c r="E106" t="n">
-        <v>314217.992904186</v>
+        <v>314305.3838743096</v>
       </c>
       <c r="F106" t="n">
-        <v>314473.4090893485</v>
+        <v>314522.0430539203</v>
       </c>
       <c r="G106" t="n">
-        <v>1.000812863015265</v>
+        <v>1.000689326975377</v>
       </c>
       <c r="H106" t="n">
-        <v>374792.5599419815</v>
+        <v>375003.9535791682</v>
       </c>
       <c r="I106" t="n">
-        <v>383022.4092823857</v>
+        <v>383143.322047335</v>
       </c>
       <c r="J106" t="n">
-        <v>145365.2066726624</v>
+        <v>145457.0160335457</v>
       </c>
       <c r="K106" t="n">
         <v>96277.61981183944</v>
@@ -10227,22 +10227,22 @@
         <v>390277.17</v>
       </c>
       <c r="E107" t="n">
-        <v>320188.1347693655</v>
+        <v>320277.1861679215</v>
       </c>
       <c r="F107" t="n">
-        <v>320762.8772711355</v>
+        <v>320686.6750977772</v>
       </c>
       <c r="G107" t="n">
-        <v>1.001795014990746</v>
+        <v>1.001278545421094</v>
       </c>
       <c r="H107" t="n">
-        <v>381913.6185808791</v>
+        <v>382129.0286971724</v>
       </c>
       <c r="I107" t="n">
-        <v>390682.8574680334</v>
+        <v>390652.9311594628</v>
       </c>
       <c r="J107" t="n">
-        <v>148127.1455994429</v>
+        <v>148220.699338183</v>
       </c>
       <c r="K107" t="n">
         <v>96111.654159395</v>
@@ -10279,22 +10279,22 @@
         <v>396298.38</v>
       </c>
       <c r="E108" t="n">
-        <v>326271.7093299834</v>
+        <v>326298.3972678783</v>
       </c>
       <c r="F108" t="n">
-        <v>326857.371939287</v>
+        <v>326651.4472545958</v>
       </c>
       <c r="G108" t="n">
-        <v>1.001795014990746</v>
+        <v>1.001081985047042</v>
       </c>
       <c r="H108" t="n">
-        <v>389169.9773339158</v>
+        <v>389313.0544366792</v>
       </c>
       <c r="I108" t="n">
-        <v>398105.831759926</v>
+        <v>397919.0756790288</v>
       </c>
       <c r="J108" t="n">
-        <v>150941.5613658323</v>
+        <v>151007.2484857408</v>
       </c>
       <c r="K108" t="n">
         <v>95677.8326172236</v>
@@ -10331,22 +10331,22 @@
         <v>403085.39</v>
       </c>
       <c r="E109" t="n">
-        <v>333123.415225913</v>
+        <v>333085.4039310502</v>
       </c>
       <c r="F109" t="n">
-        <v>334048.2341219513</v>
+        <v>333739.7836600206</v>
       </c>
       <c r="G109" t="n">
-        <v>1.002776205015223</v>
+        <v>1.001964600433545</v>
       </c>
       <c r="H109" t="n">
-        <v>397342.546857928</v>
+        <v>397410.765968962</v>
       </c>
       <c r="I109" t="n">
-        <v>406864.1600586444</v>
+        <v>406553.9196212637</v>
       </c>
       <c r="J109" t="n">
-        <v>154111.3341545148</v>
+        <v>154148.1992542442</v>
       </c>
       <c r="K109" t="n">
         <v>95310.96892028471</v>
@@ -10383,22 +10383,22 @@
         <v>410879.59</v>
       </c>
       <c r="E110" t="n">
-        <v>340785.253776109</v>
+        <v>340879.6023830368</v>
       </c>
       <c r="F110" t="n">
-        <v>341731.3435067562</v>
+        <v>341549.2945976651</v>
       </c>
       <c r="G110" t="n">
-        <v>1.002776205015223</v>
+        <v>1.001964600433545</v>
       </c>
       <c r="H110" t="n">
-        <v>406481.4254356603</v>
+        <v>406710.1778926358</v>
       </c>
       <c r="I110" t="n">
-        <v>416222.0357399932</v>
+        <v>416067.2813404013</v>
       </c>
       <c r="J110" t="n">
-        <v>157655.8948400686</v>
+        <v>157755.2671167935</v>
       </c>
       <c r="K110" t="n">
         <v>94842.71303333271</v>
@@ -10435,22 +10435,22 @@
         <v>419299.32</v>
       </c>
       <c r="E111" t="n">
-        <v>349304.8851205116</v>
+        <v>349299.3285618978</v>
       </c>
       <c r="F111" t="n">
-        <v>350616.3584379319</v>
+        <v>350258.8016099056</v>
       </c>
       <c r="G111" t="n">
-        <v>1.003754523264018</v>
+        <v>1.002746850536352</v>
       </c>
       <c r="H111" t="n">
-        <v>416643.4610715518</v>
+        <v>416755.9192865839</v>
       </c>
       <c r="I111" t="n">
-        <v>427043.8086692331</v>
+        <v>426676.9970145815</v>
       </c>
       <c r="J111" t="n">
-        <v>161597.2922110703</v>
+        <v>161651.8222145783</v>
       </c>
       <c r="K111" t="n">
         <v>94463.25767815557</v>
@@ -10487,22 +10487,22 @@
         <v>429254.35</v>
       </c>
       <c r="E112" t="n">
-        <v>359085.421903886</v>
+        <v>359254.3594259119</v>
       </c>
       <c r="F112" t="n">
-        <v>360784.2328326319</v>
+        <v>360381.2809764318</v>
       </c>
       <c r="G112" t="n">
-        <v>1.004730938169917</v>
+        <v>1.00313683472713</v>
       </c>
       <c r="H112" t="n">
-        <v>428309.4779815552</v>
+        <v>428633.4629862515</v>
       </c>
       <c r="I112" t="n">
-        <v>439428.0791206408</v>
+        <v>439007.9622283029</v>
       </c>
       <c r="J112" t="n">
-        <v>166122.0163929803</v>
+        <v>166258.8991476938</v>
       </c>
       <c r="K112" t="n">
         <v>94420.73460926655</v>
@@ -10539,22 +10539,22 @@
         <v>439600.88</v>
       </c>
       <c r="E113" t="n">
-        <v>369498.8991390986</v>
+        <v>369600.8849773781</v>
       </c>
       <c r="F113" t="n">
-        <v>371246.9755847781</v>
+        <v>370940.4525090413</v>
       </c>
       <c r="G113" t="n">
-        <v>1.004730938169917</v>
+        <v>1.003624362348984</v>
       </c>
       <c r="H113" t="n">
-        <v>440730.4528430203</v>
+        <v>440978.1067202555</v>
       </c>
       <c r="I113" t="n">
-        <v>452171.4934151393</v>
+        <v>451870.8955215922</v>
       </c>
       <c r="J113" t="n">
-        <v>170939.5548683767</v>
+        <v>171047.1554431474</v>
       </c>
       <c r="K113" t="n">
         <v>93961.68422360416</v>
@@ -10591,22 +10591,22 @@
         <v>450319.31</v>
       </c>
       <c r="E114" t="n">
-        <v>380214.3672141324</v>
+        <v>380319.310641722</v>
       </c>
       <c r="F114" t="n">
-        <v>382755.6318279062</v>
+        <v>382365.4184463198</v>
       </c>
       <c r="G114" t="n">
-        <v>1.006683767981715</v>
+        <v>1.005379973478458</v>
       </c>
       <c r="H114" t="n">
-        <v>453511.6359754678</v>
+        <v>453766.4718151429</v>
       </c>
       <c r="I114" t="n">
-        <v>466188.8097110086</v>
+        <v>465788.5191036572</v>
       </c>
       <c r="J114" t="n">
-        <v>175896.8019595596</v>
+        <v>176007.5229509987</v>
       </c>
       <c r="K114" t="n">
         <v>94252.79772593097</v>
@@ -10643,22 +10643,22 @@
         <v>463174.1</v>
       </c>
       <c r="E115" t="n">
-        <v>393141.655699413</v>
+        <v>393174.1033414122</v>
       </c>
       <c r="F115" t="n">
-        <v>395003.8120463992</v>
+        <v>394754.0580039805</v>
       </c>
       <c r="G115" t="n">
-        <v>1.004736604020435</v>
+        <v>1.004018460649216</v>
       </c>
       <c r="H115" t="n">
-        <v>468931.0315986337</v>
+        <v>469103.7785624947</v>
       </c>
       <c r="I115" t="n">
-        <v>481106.8516217609</v>
+        <v>480880.0671226157</v>
       </c>
       <c r="J115" t="n">
-        <v>181877.2932261846</v>
+        <v>181956.5772267424</v>
       </c>
       <c r="K115" t="n">
         <v>95387.73178112155</v>
@@ -10695,22 +10695,22 @@
         <v>473317.99</v>
       </c>
       <c r="E116" t="n">
-        <v>403363.3387475977</v>
+        <v>403317.9952076207</v>
       </c>
       <c r="F116" t="n">
-        <v>405273.9111596055</v>
+        <v>404899.2372946828</v>
       </c>
       <c r="G116" t="n">
-        <v>1.004736604020435</v>
+        <v>1.00392058402018</v>
       </c>
       <c r="H116" t="n">
-        <v>481123.2384201982</v>
+        <v>481206.6560494071</v>
       </c>
       <c r="I116" t="n">
-        <v>493615.6297639267</v>
+        <v>493238.6848476669</v>
       </c>
       <c r="J116" t="n">
-        <v>186606.1028500654</v>
+        <v>186651.0569191924</v>
       </c>
       <c r="K116" t="n">
         <v>96036.64674223015</v>
@@ -10747,22 +10747,22 @@
         <v>481989.33</v>
       </c>
       <c r="E117" t="n">
-        <v>411833.9688612972</v>
+        <v>411989.3321045846</v>
       </c>
       <c r="F117" t="n">
-        <v>414595.2111162764</v>
+        <v>414130.9399050015</v>
       </c>
       <c r="G117" t="n">
-        <v>1.006704746241826</v>
+        <v>1.005198211782516</v>
       </c>
       <c r="H117" t="n">
-        <v>491226.8264270223</v>
+        <v>491552.5991544694</v>
       </c>
       <c r="I117" t="n">
-        <v>504968.789248497</v>
+        <v>504484.5268621937</v>
       </c>
       <c r="J117" t="n">
-        <v>190524.8310099168</v>
+        <v>190664.054642955</v>
       </c>
       <c r="K117" t="n">
         <v>96070.71904337834</v>
@@ -10799,22 +10799,22 @@
         <v>489775.93</v>
       </c>
       <c r="E118" t="n">
-        <v>419658.8142696618</v>
+        <v>419775.9304813612</v>
       </c>
       <c r="F118" t="n">
-        <v>422887.115338602</v>
+        <v>422496.3848910826</v>
       </c>
       <c r="G118" t="n">
-        <v>1.007692680242064</v>
+        <v>1.006480729866055</v>
       </c>
       <c r="H118" t="n">
-        <v>500560.1361291357</v>
+        <v>500842.9432784888</v>
       </c>
       <c r="I118" t="n">
-        <v>515068.1650334669</v>
+        <v>514675.11430481</v>
       </c>
       <c r="J118" t="n">
-        <v>194144.8027991052</v>
+        <v>194267.6052757069</v>
       </c>
       <c r="K118" t="n">
         <v>96288.82564092237</v>
@@ -10851,22 +10851,22 @@
         <v>498633.202123</v>
       </c>
       <c r="E119" t="n">
-        <v>428471.6493693247</v>
+        <v>428633.2026145178</v>
       </c>
       <c r="F119" t="n">
-        <v>432190.6318760513</v>
+        <v>431918.0542741537</v>
       </c>
       <c r="G119" t="n">
-        <v>1.008679646628197</v>
+        <v>1.007663549252833</v>
       </c>
       <c r="H119" t="n">
-        <v>511071.8989878476</v>
+        <v>511410.7293816649</v>
       </c>
       <c r="I119" t="n">
-        <v>526399.6646642032</v>
+        <v>526152.3693538073</v>
       </c>
       <c r="J119" t="n">
-        <v>198221.8436578864</v>
+        <v>198366.6517470242</v>
       </c>
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr"/>
@@ -10924,7 +10924,7 @@
         <v>0.1100999858071403</v>
       </c>
       <c r="D2" t="n">
-        <v>0.11</v>
+        <v>0.1101</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -10943,7 +10943,7 @@
         <v>0.08829998274969819</v>
       </c>
       <c r="D3" t="n">
-        <v>0.08800000000000001</v>
+        <v>0.0883</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -10962,7 +10962,7 @@
         <v>0.04180000009665052</v>
       </c>
       <c r="D4" t="n">
-        <v>0.042</v>
+        <v>0.0418</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -10981,7 +10981,7 @@
         <v>0.04579999278228919</v>
       </c>
       <c r="D5" t="n">
-        <v>0.046</v>
+        <v>0.0458</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -11000,7 +11000,7 @@
         <v>0.04029998613466979</v>
       </c>
       <c r="D6" t="n">
-        <v>0.04</v>
+        <v>0.0403</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -11019,7 +11019,7 @@
         <v>0.04170001027115888</v>
       </c>
       <c r="D7" t="n">
-        <v>0.042</v>
+        <v>0.0417</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -11038,7 +11038,7 @@
         <v>0.03469998595288093</v>
       </c>
       <c r="D8" t="n">
-        <v>0.035</v>
+        <v>0.0347</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -11057,7 +11057,7 @@
         <v>0.0269000035126794</v>
       </c>
       <c r="D9" t="n">
-        <v>0.027</v>
+        <v>0.0269</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -11076,7 +11076,7 @@
         <v>0.02430000050847703</v>
       </c>
       <c r="D10" t="n">
-        <v>0.024</v>
+        <v>0.0243</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -11114,7 +11114,7 @@
         <v>0.02209999395795847</v>
       </c>
       <c r="D12" t="n">
-        <v>0.022</v>
+        <v>0.0221</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
@@ -11152,7 +11152,7 @@
         <v>0.03730000175284753</v>
       </c>
       <c r="D14" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.0373</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
@@ -11171,7 +11171,7 @@
         <v>0.02779999199950733</v>
       </c>
       <c r="D15" t="n">
-        <v>0.028</v>
+        <v>0.0278</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
@@ -11209,7 +11209,7 @@
         <v>0.01620001423237682</v>
       </c>
       <c r="D17" t="n">
-        <v>0.016</v>
+        <v>0.0162</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
@@ -11247,7 +11247,7 @@
         <v>0.01879999751465267</v>
       </c>
       <c r="D19" t="n">
-        <v>0.019</v>
+        <v>0.0188</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
@@ -11266,7 +11266,7 @@
         <v>0.02080001132705589</v>
       </c>
       <c r="D20" t="n">
-        <v>0.021</v>
+        <v>0.0208</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
@@ -11285,7 +11285,7 @@
         <v>0.02340000562618494</v>
       </c>
       <c r="D21" t="n">
-        <v>0.023</v>
+        <v>0.0234</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
@@ -11304,7 +11304,7 @@
         <v>0.0247000121069143</v>
       </c>
       <c r="D22" t="n">
-        <v>0.025</v>
+        <v>0.0247</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
@@ -11323,7 +11323,7 @@
         <v>0.02849999822501803</v>
       </c>
       <c r="D23" t="n">
-        <v>0.028</v>
+        <v>0.0285</v>
       </c>
       <c r="E23" t="b">
         <v>1</v>
@@ -11342,7 +11342,7 @@
         <v>0.02880001313832392</v>
       </c>
       <c r="D24" t="n">
-        <v>0.029</v>
+        <v>0.0288</v>
       </c>
       <c r="E24" t="b">
         <v>1</v>
@@ -11380,7 +11380,7 @@
         <v>0.03379999295854841</v>
       </c>
       <c r="D26" t="n">
-        <v>0.034</v>
+        <v>0.0338</v>
       </c>
       <c r="E26" t="b">
         <v>1</v>
@@ -11399,7 +11399,7 @@
         <v>0.02579999547274348</v>
       </c>
       <c r="D27" t="n">
-        <v>0.026</v>
+        <v>0.0258</v>
       </c>
       <c r="E27" t="b">
         <v>1</v>
@@ -11418,7 +11418,7 @@
         <v>0.02150000797137763</v>
       </c>
       <c r="D28" t="n">
-        <v>0.021</v>
+        <v>0.0215</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
@@ -11437,7 +11437,7 @@
         <v>0.01890000403651215</v>
       </c>
       <c r="D29" t="n">
-        <v>0.019</v>
+        <v>0.0189</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
@@ -11456,7 +11456,7 @@
         <v>0.0210999999999999</v>
       </c>
       <c r="D30" t="n">
-        <v>0.021</v>
+        <v>0.0211</v>
       </c>
       <c r="E30" t="b">
         <v>1</v>
@@ -11527,13 +11527,13 @@
         <v>2555298.3</v>
       </c>
       <c r="C3" t="n">
-        <v>0.999099099099099</v>
+        <v>0.999189262228628</v>
       </c>
       <c r="D3" t="n">
-        <v>-2302.070540540801</v>
+        <v>-2071.676848932589</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.09009009009010027</v>
+        <v>-0.08107377713719721</v>
       </c>
     </row>
     <row r="4">
@@ -11546,13 +11546,13 @@
         <v>4202722.9</v>
       </c>
       <c r="C4" t="n">
-        <v>1.003690547164812</v>
+        <v>1.00368804692487</v>
       </c>
       <c r="D4" t="n">
-        <v>15510.34708308401</v>
+        <v>15499.83926742532</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3690547164811653</v>
+        <v>0.3688046924869903</v>
       </c>
     </row>
     <row r="5">
@@ -11565,13 +11565,13 @@
         <v>3010772</v>
       </c>
       <c r="C5" t="n">
-        <v>1.001764077784457</v>
+        <v>1.00156852906805</v>
       </c>
       <c r="D5" t="n">
-        <v>5311.235999264426</v>
+        <v>4722.483399271857</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1764077784456752</v>
+        <v>0.1568529068050273</v>
       </c>
     </row>
     <row r="6">
@@ -11584,13 +11584,13 @@
         <v>3118531.9</v>
       </c>
       <c r="C6" t="n">
-        <v>1.002721787227845</v>
+        <v>1.002909316924902</v>
       </c>
       <c r="D6" t="n">
-        <v>8487.980295047535</v>
+        <v>9072.797637515874</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2721787227845107</v>
+        <v>0.2909316924901706</v>
       </c>
     </row>
     <row r="7">
@@ -11603,13 +11603,13 @@
         <v>3256710.2</v>
       </c>
       <c r="C7" t="n">
-        <v>1.003685942792487</v>
+        <v>1.003584157376548</v>
       </c>
       <c r="D7" t="n">
-        <v>12004.04748890932</v>
+        <v>11672.56188660854</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3685942792487129</v>
+        <v>0.3584157376547825</v>
       </c>
     </row>
     <row r="8">
@@ -11622,13 +11622,13 @@
         <v>3334485.5</v>
       </c>
       <c r="C8" t="n">
-        <v>1.003685942792487</v>
+        <v>1.004162203353725</v>
       </c>
       <c r="D8" t="n">
-        <v>12290.72279537858</v>
+        <v>13878.80673104802</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3685942792487351</v>
+        <v>0.4162203353725191</v>
       </c>
     </row>
     <row r="9">
@@ -11641,13 +11641,13 @@
         <v>3505778</v>
       </c>
       <c r="C9" t="n">
-        <v>1.002716197920224</v>
+        <v>1.003871057455391</v>
       </c>
       <c r="D9" t="n">
-        <v>9522.386912367581</v>
+        <v>13571.06806384677</v>
       </c>
       <c r="E9" t="n">
-        <v>0.271619792022415</v>
+        <v>0.3871057455391291</v>
       </c>
     </row>
     <row r="10">
@@ -11660,13 +11660,13 @@
         <v>5335814.7</v>
       </c>
       <c r="C10" t="n">
-        <v>1.001739843297128</v>
+        <v>1.003382270301114</v>
       </c>
       <c r="D10" t="n">
-        <v>9283.481440510017</v>
+        <v>18047.16759205596</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1739843297127619</v>
+        <v>0.338227030111371</v>
       </c>
     </row>
     <row r="11">
@@ -11679,13 +11679,13 @@
         <v>3762351.2</v>
       </c>
       <c r="C11" t="n">
-        <v>1.001739843297128</v>
+        <v>1.002990438896134</v>
       </c>
       <c r="D11" t="n">
-        <v>6545.901516760054</v>
+        <v>11251.08136939783</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1739843297127619</v>
+        <v>0.2990438896134373</v>
       </c>
     </row>
     <row r="12">
@@ -11698,13 +11698,13 @@
         <v>3863750.9</v>
       </c>
       <c r="C12" t="n">
-        <v>1.001739843297128</v>
+        <v>1.003088101061558</v>
       </c>
       <c r="D12" t="n">
-        <v>6722.321105135805</v>
+        <v>11931.65325588393</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1739843297127619</v>
+        <v>0.3088101061557547</v>
       </c>
     </row>
     <row r="13">
@@ -11717,13 +11717,13 @@
         <v>3945383.3</v>
       </c>
       <c r="C13" t="n">
-        <v>1.001739843297128</v>
+        <v>1.003284380897398</v>
       </c>
       <c r="D13" t="n">
-        <v>6864.348689104247</v>
+        <v>12958.14154343273</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1739843297127619</v>
+        <v>0.3284380897397909</v>
       </c>
     </row>
     <row r="14">
@@ -11736,13 +11736,13 @@
         <v>4047468.9</v>
       </c>
       <c r="C14" t="n">
-        <v>1.002718104862847</v>
+        <v>1.004460104781262</v>
       </c>
       <c r="D14" t="n">
-        <v>11001.44489931318</v>
+        <v>18052.13539289933</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2718104862847293</v>
+        <v>0.446010478126202</v>
       </c>
     </row>
     <row r="15">
@@ -11755,13 +11755,13 @@
         <v>4224941.8</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9998172810300717</v>
+        <v>1.00116774542885</v>
       </c>
       <c r="D15" t="n">
-        <v>-771.9770137029119</v>
+        <v>4933.656474108735</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0182718969928275</v>
+        <v>0.1167745428850342</v>
       </c>
     </row>
     <row r="16">
@@ -11774,13 +11774,13 @@
         <v>6196115</v>
       </c>
       <c r="C16" t="n">
-        <v>0.9988446961263459</v>
+        <v>0.999901430903595</v>
       </c>
       <c r="D16" t="n">
-        <v>-7158.395661106555</v>
+        <v>-610.7454567717356</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1155303873654145</v>
+        <v>-0.009856909640504341</v>
       </c>
     </row>
     <row r="17">
@@ -11793,13 +11793,13 @@
         <v>4707376.6</v>
       </c>
       <c r="C17" t="n">
-        <v>0.9998287795708054</v>
+        <v>1.000393993184828</v>
       </c>
       <c r="D17" t="n">
-        <v>-805.9990418325991</v>
+        <v>1854.674298821001</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.01712204291945962</v>
+        <v>0.03939931848284672</v>
       </c>
     </row>
     <row r="18">
@@ -11812,13 +11812,13 @@
         <v>4468820.600000001</v>
       </c>
       <c r="C18" t="n">
-        <v>1.000812863015265</v>
+        <v>1.000689326975377</v>
       </c>
       <c r="D18" t="n">
-        <v>3632.538987592648</v>
+        <v>3080.478587699152</v>
       </c>
       <c r="E18" t="n">
-        <v>0.08128630152646199</v>
+        <v>0.06893269753767139</v>
       </c>
     </row>
     <row r="19">
@@ -11831,13 +11831,13 @@
         <v>4595791.5</v>
       </c>
       <c r="C19" t="n">
-        <v>1.001795014990746</v>
+        <v>1.001278545421094</v>
       </c>
       <c r="D19" t="n">
-        <v>8249.514636842903</v>
+        <v>5875.928178625489</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1795014990745969</v>
+        <v>0.1278545421093513</v>
       </c>
     </row>
     <row r="20">
@@ -11850,13 +11850,13 @@
         <v>4684325.699999999</v>
       </c>
       <c r="C20" t="n">
-        <v>1.001795014990746</v>
+        <v>1.001081985047042</v>
       </c>
       <c r="D20" t="n">
-        <v>8408.434853036602</v>
+        <v>5068.370362872677</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1795014990745969</v>
+        <v>0.10819850470416</v>
       </c>
     </row>
     <row r="21">
@@ -11869,13 +11869,13 @@
         <v>4789901.500000001</v>
       </c>
       <c r="C21" t="n">
-        <v>1.002776205015223</v>
+        <v>1.001964600433545</v>
       </c>
       <c r="D21" t="n">
-        <v>13297.74856672374</v>
+        <v>9410.242563536596</v>
       </c>
       <c r="E21" t="n">
-        <v>0.277620501522291</v>
+        <v>0.1964600433544739</v>
       </c>
     </row>
     <row r="22">
@@ -11888,13 +11888,13 @@
         <v>7386910.4</v>
       </c>
       <c r="C22" t="n">
-        <v>1.002776205015223</v>
+        <v>1.001964600433545</v>
       </c>
       <c r="D22" t="n">
-        <v>20507.57769948227</v>
+        <v>14512.32737439614</v>
       </c>
       <c r="E22" t="n">
-        <v>0.277620501522291</v>
+        <v>0.1964600433544739</v>
       </c>
     </row>
     <row r="23">
@@ -11907,13 +11907,13 @@
         <v>5077070.1</v>
       </c>
       <c r="C23" t="n">
-        <v>1.003754523264018</v>
+        <v>1.002746850536352</v>
       </c>
       <c r="D23" t="n">
-        <v>19061.97780350208</v>
+        <v>13945.9527272836</v>
       </c>
       <c r="E23" t="n">
-        <v>0.3754523264018372</v>
+        <v>0.2746850536352374</v>
       </c>
     </row>
     <row r="24">
@@ -11926,13 +11926,13 @@
         <v>5220469.1</v>
       </c>
       <c r="C24" t="n">
-        <v>1.004730938169917</v>
+        <v>1.00313683472713</v>
       </c>
       <c r="D24" t="n">
-        <v>24697.71653006334</v>
+        <v>16375.74876478736</v>
       </c>
       <c r="E24" t="n">
-        <v>0.4730938169917209</v>
+        <v>0.3136834727129667</v>
       </c>
     </row>
     <row r="25">
@@ -11945,13 +11945,13 @@
         <v>5335179.899999999</v>
       </c>
       <c r="C25" t="n">
-        <v>1.004730938169917</v>
+        <v>1.003624362348984</v>
       </c>
       <c r="D25" t="n">
-        <v>25240.40623228389</v>
+        <v>19336.62515461741</v>
       </c>
       <c r="E25" t="n">
-        <v>0.4730938169916987</v>
+        <v>0.3624362348984222</v>
       </c>
     </row>
     <row r="26">
@@ -11964,13 +11964,13 @@
         <v>5540072.899999999</v>
       </c>
       <c r="C26" t="n">
-        <v>1.006683767981715</v>
+        <v>1.005379973478458</v>
       </c>
       <c r="D26" t="n">
-        <v>37028.56186538508</v>
+        <v>29805.44527072193</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6683767981714661</v>
+        <v>0.5379973478457645</v>
       </c>
     </row>
     <row r="27">
@@ -11983,13 +11983,13 @@
         <v>5677550.100000001</v>
       </c>
       <c r="C27" t="n">
-        <v>1.004736604020435</v>
+        <v>1.004018460649216</v>
       </c>
       <c r="D27" t="n">
-        <v>26892.30662987905</v>
+        <v>22815.0116608034</v>
       </c>
       <c r="E27" t="n">
-        <v>0.4736604020434632</v>
+        <v>0.4018460649216182</v>
       </c>
     </row>
     <row r="28">
@@ -12002,13 +12002,13 @@
         <v>8664734.6</v>
       </c>
       <c r="C28" t="n">
-        <v>1.004736604020435</v>
+        <v>1.00392058402018</v>
       </c>
       <c r="D28" t="n">
-        <v>41041.41674235906</v>
+        <v>33970.82001186388</v>
       </c>
       <c r="E28" t="n">
-        <v>0.4736604020434632</v>
+        <v>0.3920584020180362</v>
       </c>
     </row>
     <row r="29">
@@ -12021,13 +12021,13 @@
         <v>6014065.1</v>
       </c>
       <c r="C29" t="n">
-        <v>1.006704746241826</v>
+        <v>1.005198211782516</v>
       </c>
       <c r="D29" t="n">
-        <v>40322.78037732417</v>
+        <v>31262.38406363963</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6704746241826376</v>
+        <v>0.5198211782516227</v>
       </c>
     </row>
     <row r="30">
@@ -12040,13 +12040,13 @@
         <v>5846619.200000001</v>
       </c>
       <c r="C30" t="n">
-        <v>1.007692680242064</v>
+        <v>1.006480729866055</v>
       </c>
       <c r="D30" t="n">
-        <v>44976.17200271099</v>
+        <v>37890.35966488782</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7692680242063821</v>
+        <v>0.6480729866054524</v>
       </c>
     </row>
   </sheetData>
@@ -12136,7 +12136,7 @@
         <v>30612285.3</v>
       </c>
       <c r="D2" t="n">
-        <v>70108.13147402066</v>
+        <v>84393.04772883977</v>
       </c>
       <c r="E2" t="n">
         <v>6537505.5</v>
@@ -12145,19 +12145,19 @@
         <v>631627.4000000004</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2290195938884075</v>
+        <v>0.2756835920670051</v>
       </c>
       <c r="H2" t="n">
-        <v>1.072398814410491</v>
+        <v>1.290905953789863</v>
       </c>
       <c r="I2" t="n">
-        <v>11.09960262553851</v>
+        <v>13.36120752976196</v>
       </c>
       <c r="J2" t="n">
         <v>584377011.02669</v>
       </c>
       <c r="K2" t="n">
-        <v>0.01199707212144569</v>
+        <v>0.01444154135710608</v>
       </c>
       <c r="L2" t="n">
         <v>5.238447906466646</v>
@@ -12174,7 +12174,7 @@
         <v>56673137.4</v>
       </c>
       <c r="D3" t="n">
-        <v>76493.45923734939</v>
+        <v>98317.94394490187</v>
       </c>
       <c r="E3" t="n">
         <v>11769218.7</v>
@@ -12183,19 +12183,19 @@
         <v>1453819.100000002</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1349730449850645</v>
+        <v>0.1734824441621647</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6499450914048303</v>
+        <v>0.8353820797373903</v>
       </c>
       <c r="I3" t="n">
-        <v>5.261552777601374</v>
+        <v>6.76273574510761</v>
       </c>
       <c r="J3" t="n">
         <v>850239798.2248749</v>
       </c>
       <c r="K3" t="n">
-        <v>0.008996692391611395</v>
+        <v>0.01156355467600663</v>
       </c>
       <c r="L3" t="n">
         <v>6.665547474762039</v>
@@ -12212,7 +12212,7 @@
         <v>47375761</v>
       </c>
       <c r="D4" t="n">
-        <v>259261.3381835077</v>
+        <v>205402.347318605</v>
       </c>
       <c r="E4" t="n">
         <v>12277683.7</v>
@@ -12221,13 +12221,13 @@
         <v>2336619.799999998</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5472446937232474</v>
+        <v>0.4335599956243553</v>
       </c>
       <c r="H4" t="n">
-        <v>2.11164698911007</v>
+        <v>1.672973113964527</v>
       </c>
       <c r="I4" t="n">
-        <v>11.09557225285465</v>
+        <v>8.79057634102926</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>

</xml_diff>

<commit_message>
Notebooks robustos a sesiones viejas de Colab y version en los ZIP
- Celda de configuracion: git fetch --depth 1 + reset --hard FETCH_HEAD en vez de
  git pull (fallaba si la copia de Colab tenia cambios locales, como dejaba el NB03
  viejo) y borra src.* de sys.modules (si no, Python seguia usando el codigo viejo ya
  importado y los ZIP mezclaban versiones). Imprime la version del repo.
- El LEEME.txt del ZIP y la hoja Notas del Excel indican el commit usado.
</commit_message>
<xml_diff>
--- a/output/IIJP_resultados.xlsx
+++ b/output/IIJP_resultados.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,19 +464,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ultimo IPC: 2026-08 | ultimo haber: 2026-09 | ultima IMIG: 2026-08 | replicas bootstrap: 500</t>
+          <t>Version del codigo (commit): cd648c2 (2026-10-06)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Niveles base dic-2016 = 100. Variaciones en %. Brechas: (1 + infl. A) / (1 + infl. B) - 1, en %.</t>
+          <t>Ultimo IPC: 2026-08 | ultimo haber: 2026-09 | ultima IMIG: 2026-08 | replicas bootstrap: 500</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
+        <is>
+          <t>Niveles base dic-2016 = 100. Variaciones en %. Brechas: (1 + infl. A) / (1 + infl. B) - 1, en %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Montos fiscales en millones de pesos corrientes. Metodologia: README y docs/ del repo github.com/santiagoriverti/IPC_jubilados.</t>
         </is>

</xml_diff>